<commit_message>
aef last bloack id title rename
</commit_message>
<xml_diff>
--- a/backend/services/libs/shared/src/templates/aef_actions_template.xlsx
+++ b/backend/services/libs/shared/src/templates/aef_actions_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AmilaDissanayake\Projects\carbon-registry-undp\carbon-registry-zim\backend\services\libs\shared\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA94FBB4-7563-47B2-AADB-9E08607A52DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3347C08B-5C67-4EB4-B990-DDF3BB4818DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4A6097B3-A9B2-43A8-BF23-64D8708A96D2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A6097B3-A9B2-43A8-BF23-64D8708A96D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Actions" sheetId="1" r:id="rId1"/>
@@ -177,9 +177,6 @@
     <t>First transfer</t>
   </si>
   <si>
-    <t>Underlying unit last block end ID</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Conversion factor </t>
     </r>
@@ -204,6 +201,9 @@
       </rPr>
       <t>(reporting Party)</t>
     </r>
+  </si>
+  <si>
+    <t>Underlying unit block last ID</t>
   </si>
 </sst>
 </file>
@@ -407,29 +407,29 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -814,95 +814,95 @@
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="18"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="14"/>
       <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
       <c r="R8" s="12"/>
-      <c r="S8" s="14" t="s">
+      <c r="S8" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="T8" s="17" t="s">
+      <c r="T8" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="U8" s="17"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="17"/>
-      <c r="Z8" s="17"/>
+      <c r="U8" s="21"/>
+      <c r="V8" s="21"/>
+      <c r="W8" s="21"/>
+      <c r="X8" s="21"/>
+      <c r="Y8" s="21"/>
+      <c r="Z8" s="21"/>
     </row>
     <row r="9" spans="1:26" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="17" t="s">
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17" t="s">
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17" t="s">
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="19" t="s">
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="15"/>
-      <c r="T9" s="20" t="s">
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20"/>
-      <c r="Y9" s="20"/>
-      <c r="Z9" s="21"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="15"/>
     </row>
     <row r="10" spans="1:26" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="11" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="22" t="s">
-        <v>37</v>
+      <c r="F10" s="16" t="s">
+        <v>38</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>21</v>
@@ -914,7 +914,7 @@
         <v>12</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>23</v>
@@ -940,7 +940,7 @@
       <c r="R10" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="S10" s="16"/>
+      <c r="S10" s="20"/>
       <c r="T10" s="11" t="s">
         <v>30</v>
       </c>

</xml_diff>